<commit_message>
fix QueryTianya hub xlsx province
</commit_message>
<xml_diff>
--- a/data-raw/data-tidy/hack-tianyan/hub/match-tianyan-tot-2024-06-hand.xlsx
+++ b/data-raw/data-tidy/hack-tianyan/hub/match-tianyan-tot-2024-06-hand.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github\techme\data-raw\data-tidy\hack-tianyan\hub\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6687D8B7-8C7C-4035-A8AB-CF3B36FBA7AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82B1198F-AAC0-4951-A708-631DDE70F410}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="143">
   <si>
     <t>index</t>
   </si>
@@ -250,10 +250,6 @@
     <t>https://www.tianyancha.com/company/466917033</t>
   </si>
   <si>
-    <t>河北省</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>廊坊市</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -293,10 +289,6 @@
     <t>0795-2525225</t>
   </si>
   <si>
-    <t>江西省</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>宜春市</t>
   </si>
   <si>
@@ -333,10 +325,6 @@
   </si>
   <si>
     <t>海南省海口市龙华区学院路4号</t>
-  </si>
-  <si>
-    <t>海南省</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>海口市</t>
@@ -1554,13 +1542,13 @@
         <v>41</v>
       </c>
       <c r="G4" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="H4" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="I4" s="2" t="s">
         <v>43</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -1568,28 +1556,28 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D5" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="C5" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="D5" s="7" t="s">
+      <c r="E5" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="F5" t="s">
+        <v>49</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="H5" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="F5" t="s">
-        <v>51</v>
-      </c>
-      <c r="G5" s="8" t="s">
+      <c r="I5" s="2" t="s">
         <v>48</v>
-      </c>
-      <c r="H5" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -1597,25 +1585,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="F6" t="s">
+        <v>54</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H6" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="D6" s="7" t="s">
+      <c r="I6" s="2" t="s">
         <v>53</v>
-      </c>
-      <c r="F6" t="s">
-        <v>57</v>
-      </c>
-      <c r="G6" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="H6" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -1629,16 +1617,19 @@
         <v>19</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="F7" t="s">
+        <v>55</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="H7" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="H7" s="2" t="s">
-        <v>61</v>
-      </c>
       <c r="I7" s="2" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -1652,19 +1643,19 @@
         <v>20</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="F8" t="s">
+        <v>59</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="H8" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="G8" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>65</v>
-      </c>
       <c r="I8" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
@@ -1678,16 +1669,19 @@
         <v>21</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="F9" t="s">
-        <v>66</v>
+        <v>63</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>43</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -1701,16 +1695,19 @@
         <v>22</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="F10" t="s">
+        <v>66</v>
+      </c>
+      <c r="G10" s="2" t="s">
         <v>69</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -1721,16 +1718,19 @@
         <v>23</v>
       </c>
       <c r="C11" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="G11" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="D11" s="7" t="s">
-        <v>74</v>
-      </c>
       <c r="H11" s="2" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -1741,13 +1741,16 @@
         <v>24</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="F12" t="s">
-        <v>79</v>
+        <v>76</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>16</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>16</v>
@@ -1758,22 +1761,25 @@
         <v>12</v>
       </c>
       <c r="B13" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="F13" t="s">
+        <v>79</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="H13" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="C13" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="D13" s="7" t="s">
+      <c r="I13" s="2" t="s">
         <v>81</v>
-      </c>
-      <c r="F13" t="s">
-        <v>82</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="I13" s="2" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
@@ -1781,22 +1787,25 @@
         <v>13</v>
       </c>
       <c r="B14" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="F14" t="s">
+        <v>83</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="H14" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="C14" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="D14" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="F14" t="s">
+      <c r="I14" s="2" t="s">
         <v>86</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="I14" s="2" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -1804,22 +1813,25 @@
         <v>14</v>
       </c>
       <c r="B15" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="F15" t="s">
+        <v>89</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="H15" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="C15" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="D15" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="F15" t="s">
-        <v>92</v>
-      </c>
-      <c r="H15" s="2" t="s">
-        <v>93</v>
-      </c>
       <c r="I15" s="2" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -1833,16 +1845,19 @@
         <v>25</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="F16" t="s">
+        <v>91</v>
+      </c>
+      <c r="G16" s="2" t="s">
         <v>94</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -1856,16 +1871,19 @@
         <v>26</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="F17" t="s">
+        <v>95</v>
+      </c>
+      <c r="G17" s="2" t="s">
         <v>98</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -1879,16 +1897,19 @@
         <v>27</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="F18" t="s">
-        <v>103</v>
+        <v>100</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>73</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -1902,16 +1923,19 @@
         <v>28</v>
       </c>
       <c r="D19" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="F19" t="s">
+        <v>103</v>
+      </c>
+      <c r="G19" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="F19" t="s">
-        <v>106</v>
-      </c>
       <c r="H19" s="2" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -1925,16 +1949,19 @@
         <v>29</v>
       </c>
       <c r="D20" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="F20" t="s">
+        <v>107</v>
+      </c>
+      <c r="G20" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="F20" t="s">
-        <v>110</v>
-      </c>
       <c r="H20" s="2" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
@@ -1948,16 +1975,19 @@
         <v>30</v>
       </c>
       <c r="D21" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="F21" t="s">
+        <v>111</v>
+      </c>
+      <c r="G21" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="F21" t="s">
-        <v>114</v>
-      </c>
       <c r="H21" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -1971,16 +2001,19 @@
         <v>31</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="F22" t="s">
-        <v>117</v>
+        <v>114</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>43</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -1994,16 +2027,19 @@
         <v>32</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="F23" t="s">
+        <v>128</v>
+      </c>
+      <c r="G23" s="2" t="s">
         <v>131</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -2017,16 +2053,19 @@
         <v>33</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="F24" t="s">
+        <v>117</v>
+      </c>
+      <c r="G24" s="2" t="s">
         <v>120</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
@@ -2040,16 +2079,19 @@
         <v>34</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="F25" t="s">
-        <v>124</v>
+        <v>121</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>69</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -2063,16 +2105,19 @@
         <v>35</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="F26" t="s">
+        <v>124</v>
+      </c>
+      <c r="G26" s="2" t="s">
         <v>127</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -2086,16 +2131,19 @@
         <v>36</v>
       </c>
       <c r="D27" s="12" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="F27" t="s">
-        <v>135</v>
+        <v>132</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>86</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -2103,22 +2151,25 @@
         <v>27</v>
       </c>
       <c r="B28" s="13" t="s">
+        <v>135</v>
+      </c>
+      <c r="C28" s="13" t="s">
+        <v>135</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="F28" t="s">
+        <v>136</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="H28" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="C28" s="13" t="s">
-        <v>138</v>
-      </c>
-      <c r="D28" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="F28" t="s">
-        <v>139</v>
-      </c>
-      <c r="H28" s="2" t="s">
-        <v>141</v>
-      </c>
       <c r="I28" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="29" spans="1:9" ht="18.75" x14ac:dyDescent="0.4">
@@ -2132,16 +2183,19 @@
         <v>37</v>
       </c>
       <c r="D29" s="14" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="F29" t="s">
+        <v>139</v>
+      </c>
+      <c r="G29" s="9" t="s">
         <v>142</v>
       </c>
       <c r="H29" s="8" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="I29" s="9" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
     <row r="35" spans="2:9" ht="16.5" x14ac:dyDescent="0.3">

</xml_diff>